<commit_message>
updated differential pair wiring
</commit_message>
<xml_diff>
--- a/Distance-Sensor-Board/PCB_Project/Project Outputs for Distance-Sensor-Board/Distance-Sensor-Board-BOM.xlsx
+++ b/Distance-Sensor-Board/PCB_Project/Project Outputs for Distance-Sensor-Board/Distance-Sensor-Board-BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd666c1b81e9ee1c/Documents/7-MIL/TerraGator/Distance-Sensor-Board/PCB_Project/Project Outputs for Distance-Sensor-Board/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{AC425DD0-2049-431C-A32C-BF804303C064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96A8714E-FF73-43C1-9C82-E216BCCA1BF1}"/>
+  <xr:revisionPtr revIDLastSave="289" documentId="8_{AC425DD0-2049-431C-A32C-BF804303C064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36103E20-91E9-438C-8674-DC2213FEE895}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{36416A99-A661-46BF-AA50-86C6B31C79BF}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{36416A99-A661-46BF-AA50-86C6B31C79BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Distance-Sensor-Board-BOM" sheetId="1" r:id="rId1"/>
@@ -1034,15 +1034,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C3046E4-8494-4591-93BE-702DEB3D5D59}">
   <dimension ref="A1:I40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="7" width="19.7109375" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="7" width="19.6640625" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>139</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="b">
         <v>1</v>
       </c>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="b">
         <v>1</v>
       </c>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="b">
         <v>1</v>
       </c>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="b">
         <v>1</v>
       </c>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="b">
         <v>1</v>
       </c>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="b">
         <v>1</v>
       </c>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I7" s="1"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="b">
         <v>1</v>
       </c>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="b">
         <v>1</v>
       </c>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="b">
         <v>1</v>
       </c>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="b">
         <v>0</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="b">
         <v>1</v>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="I12" s="1"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="b">
         <v>1</v>
       </c>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="b">
         <v>1</v>
       </c>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="I14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="b">
         <v>1</v>
       </c>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="b">
         <v>1</v>
       </c>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="b">
         <v>1</v>
       </c>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="I17" s="1"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="b">
         <v>1</v>
       </c>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="I18" s="1"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="b">
         <v>1</v>
       </c>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="b">
         <v>1</v>
       </c>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="b">
         <v>1</v>
       </c>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="b">
         <v>1</v>
       </c>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="b">
         <v>1</v>
       </c>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="b">
         <v>1</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="b">
         <v>1</v>
       </c>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="b">
         <v>1</v>
       </c>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="I26" s="1"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="b">
         <v>1</v>
       </c>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="b">
         <v>1</v>
       </c>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="b">
         <v>1</v>
       </c>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="b">
         <v>1</v>
       </c>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="b">
         <v>1</v>
       </c>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="I31" s="1"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="b">
         <v>1</v>
       </c>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="b">
         <v>1</v>
       </c>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="b">
         <v>1</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="b">
         <v>1</v>
       </c>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="I35" s="1"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="b">
         <v>1</v>
       </c>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="I36" s="1"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="b">
         <v>1</v>
       </c>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="I37" s="1"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="b">
         <v>1</v>
       </c>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="I38" s="1"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>140</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>141</v>
       </c>

</xml_diff>